<commit_message>
Estacas y barrios -La lista oficial: cada estaca con sus barrios y ramas, con su nombre de verdad
- 25 barrios y ramas en las cuatro estacas (Puerto Cabezas es distrito); los números ya guardados no se mueven.
- El barrio lleva prefijo en sus métodos (ward_villa_flor?) porque repite nombres de estaca, y hay dos Loma Verde.
- La carga busca el barrio solo entre los de la estaca de la fila; el filtro de barrio va agrupado por estaca.
- Una ficha vieja con un barrio que ya no es de su estaca no traba otros cambios: se valida al cambiar estaca o barrio.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QQ3Y64aehVHLknQVBkUnC2
</commit_message>
<xml_diff>
--- a/test/fixtures/files/formato_iglesia.xlsx
+++ b/test/fixtures/files/formato_iglesia.xlsx
@@ -327,7 +327,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:Y4"/>
+  <dimension ref="A1:Y5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
     <col width="16.5" min="1" max="1" bestFit="1" customWidth="1"/>
@@ -635,58 +635,54 @@
     <row r="4">
       <c r="A4" s="0" t="inlineStr">
         <is>
-          <t>Luis</t>
+          <t>Ana</t>
         </is>
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>Gómez</t>
+          <t>Kingsman</t>
         </is>
       </c>
       <c r="C4" s="0"/>
       <c r="D4" s="0" t="inlineStr">
         <is>
-          <t>05/08/2009</t>
+          <t>2011-01-20</t>
         </is>
       </c>
       <c r="E4" s="0" t="inlineStr">
         <is>
-          <t>Masculino</t>
+          <t>Femenino</t>
         </is>
       </c>
       <c r="F4" s="0" t="inlineStr">
         <is>
-          <t>8800 0000</t>
+          <t>8811 0000</t>
         </is>
       </c>
       <c r="G4" s="0"/>
-      <c r="H4" s="0" t="inlineStr">
-        <is>
-          <t>Ninguna</t>
-        </is>
-      </c>
+      <c r="H4" s="0"/>
       <c r="I4" s="0" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>S</t>
         </is>
       </c>
       <c r="J4" s="0"/>
       <c r="K4" s="0" t="inlineStr">
         <is>
-          <t>Ana Gómez</t>
+          <t>Rosa Kingsman</t>
         </is>
       </c>
       <c r="L4" s="0"/>
       <c r="M4" s="0" t="inlineStr">
         <is>
-          <t>8700 0000</t>
+          <t>8711 0000</t>
         </is>
       </c>
       <c r="N4" s="0"/>
       <c r="O4" s="0"/>
       <c r="P4" s="0"/>
       <c r="Q4" s="0" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="R4" s="0"/>
       <c r="S4" s="0" t="inlineStr">
@@ -701,17 +697,98 @@
       </c>
       <c r="U4" s="0" t="inlineStr">
         <is>
-          <t>Estaca León Nicaragua</t>
+          <t>Distrito Puerto Cabezas</t>
         </is>
       </c>
       <c r="V4" s="0" t="inlineStr">
         <is>
-          <t>Barrio Sutiava</t>
+          <t>Rama Loma Verde</t>
         </is>
       </c>
       <c r="W4" s="0"/>
       <c r="X4" s="0"/>
       <c r="Y4" s="0"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>Luis</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>Gómez</t>
+        </is>
+      </c>
+      <c r="C5" s="0"/>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>05/08/2009</t>
+        </is>
+      </c>
+      <c r="E5" s="0" t="inlineStr">
+        <is>
+          <t>Masculino</t>
+        </is>
+      </c>
+      <c r="F5" s="0" t="inlineStr">
+        <is>
+          <t>8800 0000</t>
+        </is>
+      </c>
+      <c r="G5" s="0"/>
+      <c r="H5" s="0" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="I5" s="0" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J5" s="0"/>
+      <c r="K5" s="0" t="inlineStr">
+        <is>
+          <t>Ana Gómez</t>
+        </is>
+      </c>
+      <c r="L5" s="0"/>
+      <c r="M5" s="0" t="inlineStr">
+        <is>
+          <t>8700 0000</t>
+        </is>
+      </c>
+      <c r="N5" s="0"/>
+      <c r="O5" s="0"/>
+      <c r="P5" s="0"/>
+      <c r="Q5" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="R5" s="0"/>
+      <c r="S5" s="0" t="inlineStr">
+        <is>
+          <t>Inscrito</t>
+        </is>
+      </c>
+      <c r="T5" s="0" t="inlineStr">
+        <is>
+          <t>Participante</t>
+        </is>
+      </c>
+      <c r="U5" s="0" t="inlineStr">
+        <is>
+          <t>Estaca León Nicaragua</t>
+        </is>
+      </c>
+      <c r="V5" s="0" t="inlineStr">
+        <is>
+          <t>Barrio Sutiava</t>
+        </is>
+      </c>
+      <c r="W5" s="0"/>
+      <c r="X5" s="0"/>
+      <c r="Y5" s="0"/>
     </row>
   </sheetData>
   <sheetCalcPr fullCalcOnLoad="1"/>

</xml_diff>